<commit_message>
Updated Test Case rationales for 50 rows
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases - New.xlsx
+++ b/Assignment 1 - Test cases - New.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="253">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -261,9 +261,6 @@
     <t>Mage router eka wada na.</t>
   </si>
   <si>
-    <t>මගේ router එක වැඩ නෑ.</t>
-  </si>
-  <si>
     <t>Neg_022</t>
   </si>
   <si>
@@ -438,9 +435,6 @@
     <t>හෙට 10:30ට meeting එක.</t>
   </si>
   <si>
-    <t>8.00am කියද්දි එන්න.</t>
-  </si>
-  <si>
     <t>Neg_039</t>
   </si>
   <si>
@@ -591,9 +585,6 @@
     <t>මෙස්සෙන්ගෙර් එකෙන් මෙස්සගෙ එකක් අwඅ.</t>
   </si>
   <si>
-    <t>SLT බිල්ල් එක ගෙwwඅඩ?</t>
-  </si>
-  <si>
     <t>මහෙල හොඩ බට්ස්මන් කෙනෙක්.</t>
   </si>
   <si>
@@ -613,13 +604,418 @@
   </si>
   <si>
     <t>8.00am කියඩ්ඩි එන්න.</t>
+  </si>
+  <si>
+    <t>Singlish input types covered</t>
+  </si>
+  <si>
+    <t>Evidence or rationale for the input type covered</t>
+  </si>
+  <si>
+    <t>ඔක්කෝම අයින් කරලා දාපන්.</t>
+  </si>
+  <si>
+    <t>සුබ දවසක් වෙවා!</t>
+  </si>
+  <si>
+    <t>කොහෙද ගියේ? මට කිව්වෙ නෑනේ</t>
+  </si>
+  <si>
+    <t>මගේ router එක වැඩ නෑ</t>
+  </si>
+  <si>
+    <t>මගෙ router එක වැඩ නෑ.</t>
+  </si>
+  <si>
+    <t>Jaffna යන්න කොච්චිය කීයටද?</t>
+  </si>
+  <si>
+    <t>Semi-Formal Professional Singlish</t>
+  </si>
+  <si>
+    <t>Uses work-related terms (like 'meeting', 'office') to see if the translator provides professional-level Sinhala equivalents.</t>
+  </si>
+  <si>
+    <t>Sentiment-Driven Fragmented Text</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Evaluates the translation of short, emotionally charged phrases to see if the core sentiment is maintained in Sinhala.</t>
+    </r>
+  </si>
+  <si>
+    <t>Evaluates the translation of short, emotionally charged phrases to see if the core sentiment is maintained in Sinhala.</t>
+  </si>
+  <si>
+    <t>Symbol-Heavy Textual Inputs</t>
+  </si>
+  <si>
+    <t>Sentiment-Driven Fragmented text Symbol-Heavy Textual Inputs</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Verifies if the presence of special characters (like @, #, !) interferes with the translation of the surrounding Singlish text.</t>
+    </r>
+  </si>
+  <si>
+    <t>Symbol-Heavy Textual Inputs ,Bilingual Code-Switched Inputs</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Examines the parsing capabilities of the tool when English nouns are embedded within Singlish sentence structures.</t>
+    </r>
+  </si>
+  <si>
+    <t>Symbol-Heavy Textual Inputs ,Phonetic Digital Contractions</t>
+  </si>
+  <si>
+    <t>Alphanumeric and Temporal Data</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tests the preservation of numerical values, time, and dates during the transliteration process to ensure data integrity.</t>
+    </r>
+  </si>
+  <si>
+    <t>Colloquial and Informal Slang</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Identifies whether the system can translate localized slang terms that do not follow formal linguistic rules.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Checks if the translator can accurately distinguish between polite requests and direct commands in a conversational setting.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Evaluates how the translation engine processes standard questioning formats to deliver accurate contextual responses.</t>
+    </r>
+  </si>
+  <si>
+    <t>Inquiry-Based Conversational Sentences , Colloquial and Informal Slang</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Assesses the model's ability to map informal short-hand script (like 'mn', 'mka', 'khmda') to their correct semantic meanings.</t>
+    </r>
+  </si>
+  <si>
+    <t>Alphanumeric and Temporal Data , Bilingual Code-Switched Inputs</t>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Verifies if the presence of special characters (like @, #, ! , $) interferes with the translation of the surrounding Singlish text.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Intentionally utilizes unconventional phonetic spellings to verify the system's robustness and error-correction logic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tests the software's ability to handle sentences where English and Singlish are integrated within a single context.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> This test case evaluates whether the system can distinguish between Singlish and pure English text, and if it correctly handles or bypasses non-Singlish inputs. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Evidence:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Don't talk with me again."</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tests the tool's ability to handle inputs that combine standard English sentences with their Sinhala script equivalents to ensure no character encoding issues occur. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Evidence:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "He is a very good person. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rationale:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> This case evaluates the translator's ability to process repeated emotional exclamations ("Ayyo ayyo") and colloquial question forms while maintaining the conversational sentiment in the Sinhala output. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Evidence:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Ayyo ayyo, monada me karanne?"</t>
+    </r>
+  </si>
+  <si>
+    <t>හෙට 10.30ට මීටින්ග් එක</t>
+  </si>
+  <si>
+    <t xml:space="preserve">හෙට  මේ 1ස්ට්,so ඔක්කොම ඔෆ්ෆිස නිවාඩු </t>
+  </si>
+  <si>
+    <t>Inquiry-Based Conversational Sentences , Colloquial Interrogative Sentences</t>
+  </si>
+  <si>
+    <t>Directive and Command Phrases , Colloquial Interrogative Sentences</t>
+  </si>
+  <si>
+    <t>Symbol-Heavy Textual Inputs , Colloquial Interrogative Sentences , Colloquial Interrogative Sentences</t>
+  </si>
+  <si>
+    <t>Bilingual Code-Switched Inputs , Colloquial Interrogative Sentences</t>
+  </si>
+  <si>
+    <t>Phonetic Digital Contractions , Colloquial Interrogative Sentences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phonetic Digital Contractions </t>
+  </si>
+  <si>
+    <t>Emotional Exclamations &amp; Informal Interrogatives , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Colloquial and Informal Slang , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Inquiry-Based Conversational Sentences , Sentiment-Driven Fragmented Text , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Sentiment-Driven Fragmented Text , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Phonetic Digital Contractions , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Inquiry-Based Conversational Sentences , Phonetic Digital Contractions , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Bilingual Code-Switched Inputs , Phonetic Script Contractions , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Hybrid English-Sinhala Input , Phonetic Script Contractions</t>
+  </si>
+  <si>
+    <t>Full English Sentence Input , Loanword Transliteration Patterns</t>
+  </si>
+  <si>
+    <t>Bilingual Code-Switched Inputs , Loanword Transliteration Patterns</t>
+  </si>
+  <si>
+    <t>Code-Mixed Linguistic Patterns , Loanword Transliteration Patterns</t>
+  </si>
+  <si>
+    <t>Non-Standard Script Variants , Alphanumeric Data Handling</t>
+  </si>
+  <si>
+    <t>Bilingual Code-Switched Inputs , Alphanumeric Data Handling</t>
+  </si>
+  <si>
+    <t>Inquiry-Based Conversational Sentences , Alphanumeric Data Handling</t>
+  </si>
+  <si>
+    <t>Alphanumeric and Temporal Data , Alphanumeric Data Handling</t>
+  </si>
+  <si>
+    <t>Symbol-Heavy Textual Inputs , Alphanumeric Data Handling</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -673,6 +1069,28 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -710,7 +1128,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -729,17 +1147,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1021,40 +1454,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="40.85546875" customWidth="1"/>
     <col min="4" max="4" width="42.7109375" customWidth="1"/>
     <col min="5" max="5" width="43.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="7" max="7" width="39" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" customWidth="1"/>
     <col min="9" max="10" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="G1" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1066,15 +1506,21 @@
       <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>178</v>
+      <c r="E2" s="17" t="s">
+        <v>176</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="G2" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -1092,9 +1538,15 @@
       <c r="F3" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="G3" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1106,15 +1558,21 @@
       <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>12</v>
+      <c r="E4" s="8" t="s">
+        <v>18</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="G4" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -1124,17 +1582,23 @@
         <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>18</v>
-      </c>
       <c r="F5" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="G5" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -1146,15 +1610,21 @@
       <c r="D6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>22</v>
+      <c r="E6" s="13" t="s">
+        <v>29</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="G6" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1166,15 +1636,21 @@
       <c r="D7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>29</v>
+      <c r="E7" s="13" t="s">
+        <v>198</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="G7" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -1187,14 +1663,20 @@
         <v>32</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="G8" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -1207,14 +1689,20 @@
         <v>35</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="G9" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -1227,14 +1715,20 @@
         <v>39</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="G10" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -1246,15 +1740,21 @@
       <c r="D11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>39</v>
+      <c r="E11" s="13" t="s">
+        <v>47</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="G11" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>44</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -1267,14 +1767,20 @@
         <v>46</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="G12" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>48</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -1286,15 +1792,21 @@
       <c r="D13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>51</v>
+      <c r="E13" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="G13" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -1307,14 +1819,20 @@
         <v>54</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>50</v>
+        <v>199</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="G14" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>55</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1332,9 +1850,15 @@
       <c r="F15" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="G15" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>59</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -1347,14 +1871,20 @@
         <v>61</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="G16" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1367,14 +1897,20 @@
         <v>64</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="G17" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>66</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -1386,15 +1922,21 @@
       <c r="D18" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>64</v>
+      <c r="E18" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="G18" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
         <v>69</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -1406,15 +1948,21 @@
       <c r="D19" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>72</v>
+      <c r="E19" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="G19" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>73</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -1427,14 +1975,20 @@
         <v>74</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="G20" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>75</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -1447,14 +2001,20 @@
         <v>76</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+      <c r="G21" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>78</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -1464,593 +2024,773 @@
         <v>79</v>
       </c>
       <c r="D22" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>81</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="13" t="s">
         <v>83</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>84</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>85</v>
+      <c r="G23" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>87</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>88</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="E25" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>91</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
         <v>93</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
-        <v>94</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>96</v>
-      </c>
       <c r="E27" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>98</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>100</v>
-      </c>
       <c r="E28" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
         <v>101</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>102</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="E29" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>105</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>106</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D30" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="E30" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>109</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12" t="s">
-        <v>110</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="E31" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>113</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>114</v>
+      <c r="G31" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>113</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="E32" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
-        <v>117</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D33" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="E33" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
+      <c r="B34" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="C34" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="E34" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>124</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="E35" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="10" t="s">
         <v>126</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>127</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C36" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="E36" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
         <v>129</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>130</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="E37" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>133</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C38" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="E38" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
         <v>135</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>136</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="E39" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
         <v>138</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>140</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>143</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
-        <v>144</v>
+      <c r="G40" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="10" t="s">
+        <v>142</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="12" t="s">
-        <v>147</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C42" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>148</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>150</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
-        <v>151</v>
+      <c r="G42" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="10" t="s">
+        <v>149</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H43" s="15" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C44" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="H44" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
-        <v>157</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="H45" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="12" t="s">
-        <v>160</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C46" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H46" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="12" t="s">
-        <v>163</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C47" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H47" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="10" t="s">
         <v>164</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C48" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="H48" s="16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="H49" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="10" t="s">
         <v>170</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="12" t="s">
-        <v>172</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="H50" s="15" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
         <v>173</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="12" t="s">
-        <v>175</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>19</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H51" s="15" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2059,6 +2799,6 @@
     <hyperlink ref="D47" r:id="rId2" display="https://www.test.com/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>